<commit_message>
Add --registry flag to fetch_transcripts; mark batch 2 channels as Yes
</commit_message>
<xml_diff>
--- a/rubrics/Dataset_Channel_Registry_Batch2.xlsx
+++ b/rubrics/Dataset_Channel_Registry_Batch2.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix broken channel URLs and fetch remaining 7 Batch 2 channels
The registry's @handles for several Batch 2 channels no longer resolved
to the correct YouTube channel, causing the fetcher's search fallback to
silently match unrelated decoy channels (0 results). Replaced those URLs
with verified channel IDs (Check Point Research, Rapid7, Prodaft,
ReliaQuest, HuskyHacks, SecTor, Claroty, Risky Business, Darknet Diaries,
Nextron Systems) and fetched transcripts for the ones with matching
ransomware content: C52, C55, C58, C65, C86, C91, C93.

Also marked C73, C79, C81, and C95 as Included=No — no dedicated YouTube
channel could be found for them via handle lookup or name search.
</commit_message>
<xml_diff>
--- a/rubrics/Dataset_Channel_Registry_Batch2.xlsx
+++ b/rubrics/Dataset_Channel_Registry_Batch2.xlsx
@@ -521,8 +521,6 @@
           <t>Threat briefings, ransomware family deep dives</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>SentinelLabs publishes detailed ransomware family reports; strong RaaS and affiliate model coverage.</t>
@@ -547,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@CheckPointSoftware</t>
+          <t>https://www.youtube.com/channel/UCXnlgfiXZQm1sbxMzU-8ZKA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -570,8 +568,6 @@
           <t>Threat briefings, actor profiling, family breakdowns</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>CPR produces frequent RaaS and ransomware group analyses; technically detailed.</t>
@@ -619,8 +615,6 @@
           <t>Threat briefings, attribution research, affiliate tracking</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Strong ransomware attribution and affiliate tracking content; vendor bias but technically solid.</t>
@@ -668,8 +662,6 @@
           <t>IR case studies, adversary simulation research</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Formerly F-Secure; deep IR and adversary simulation research with strong technical credibility.</t>
@@ -694,7 +686,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@Rapid7</t>
+          <t>https://www.youtube.com/channel/UCnctXOUIeRFu1BR5O0W5e9w</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -717,8 +709,6 @@
           <t>Threat briefings, exploitation research, vulnerability analysis</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>Strong on initial access exploitation used by ransomware operators; AttackerKB content relevant.</t>
@@ -766,8 +756,6 @@
           <t>Ransomware family analyses, threat intel reports</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Ransomware-focused vendor; Malwarebytes ThreatDown publishes regular family breakdowns.</t>
@@ -815,8 +803,6 @@
           <t>Actor attribution, ransomware affiliate profiling, dark web intel</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>Strong CIS/Russia-nexus ransomware actor coverage; unique dark web and affiliate intel perspective.</t>
@@ -841,7 +827,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@Prodaft</t>
+          <t>https://www.youtube.com/channel/UCdVNTCZJ_KctZPiINLX1wvg</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -864,8 +850,6 @@
           <t>Threat actor deep dives, ransomware group infiltration reports</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Publishes rare inside-access reports on ransomware group infrastructure; highly technical.</t>
@@ -913,8 +897,6 @@
           <t>Threat briefings, IOC analysis, weekly threat roundups</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>Regular threat intelligence briefings; useful for IOC and campaign tracking context.</t>
@@ -962,8 +944,6 @@
           <t>Incident response case studies, ransomware trends</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>Major IR consulting firm; quarterly threat landscape reports with strong ransomware focus.</t>
@@ -1011,8 +991,6 @@
           <t>Technical research talks, malware analysis</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>Research-oriented security consultancy; publishes detailed vulnerability and malware research.</t>
@@ -1060,8 +1038,6 @@
           <t>Ransomware family analyses, decryptor releases, trend reports</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>Exclusively ransomware-focused vendor; one of the leading sources for family-level technical detail and decryptor development.</t>
@@ -1109,8 +1085,6 @@
           <t>Malware genetic analysis, code reuse tracking, family lineage</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>Unique code-similarity approach to malware attribution; valuable for ransomware lineage and shared tooling across families.</t>
@@ -1158,8 +1132,6 @@
           <t>Dark web monitoring, ransomware leak site tracking, actor intelligence</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>Specialises in external threat intelligence including ransomware extortion sites and threat actor communications.</t>
@@ -1184,7 +1156,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@ReliaQuest</t>
+          <t>https://www.youtube.com/channel/UCdPuTyaN5bU3_GmCNFgzl3Q</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1207,8 +1179,6 @@
           <t>MDR case studies, threat briefings, ransomware trend reports</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>MDR platform vendor with regular ransomware coverage; useful for detection and response perspectives.</t>
@@ -1256,8 +1226,6 @@
           <t>Threat intel reports, IR case studies, active defence content</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>Practitioner-heavy MDR firm; publishes threat intel alongside IR and detection content.</t>
@@ -1305,8 +1273,6 @@
           <t>Memory forensics, disk triage, DFIR walkthroughs</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>Richard Davis; one of the highest-quality practitioner DFIR channels. Deep technical walkthroughs of tools and artefacts used in ransomware intrusions.</t>
@@ -1331,7 +1297,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@HuskyHacks</t>
+          <t>https://www.youtube.com/channel/UCtJgZIyoZ0wIKEzctj_8pZQ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1354,8 +1320,6 @@
           <t>Malware analysis, offensive tool walkthroughs</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
           <t>Well-structured malware analysis content; useful for understanding attacker tooling used alongside ransomware.</t>
@@ -1403,8 +1367,6 @@
           <t>Attack chain walkthroughs, red team techniques, IR fundamentals</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>The Cyber Mentor; large audience with solid coverage of techniques used in ransomware intrusion chains (credential access, lateral movement).</t>
@@ -1452,8 +1414,6 @@
           <t>Malware reverse engineering, unpacking, analysis walkthroughs</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>Detailed static and dynamic malware analysis; useful for ransomware encryption and dropper analysis.</t>
@@ -1501,8 +1461,6 @@
           <t>Live malware detonations, ransomware behaviour analysis</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>Interactive sandbox vendor; publishes ransomware execution walkthroughs with process tree and network activity detail.</t>
@@ -1550,8 +1508,6 @@
           <t>Cloud IR case studies, ransomware in cloud environments</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>Cloud-native DFIR vendor; unique coverage of ransomware targeting AWS, Azure, and GCP environments.</t>
@@ -1599,16 +1555,14 @@
           <t>ATT&amp;CK detection engineering, threat hunting, Jupyter-based analysis</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Roberto Rodriguez; MITRE ATT&amp;CK contributor. Excellent detection-layer content aligned with ransomware tactic coverage.</t>
+          <t>Roberto Rodriguez; MITRE ATT&amp;CK contributor. Excellent detection-layer content aligned with ransomware tactic coverage. [EXCLUDED: no dedicated YouTube channel found via API handle lookup or name search as of 2026-08-11 — likely hosted only on other platforms/conference archives.]</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1648,8 +1602,6 @@
           <t>Research talks, malware family analyses, threat actor profiling</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>Dedicated anti-malware/threat intelligence conference; among the highest ransomware content density of any conference channel.</t>
@@ -1697,8 +1649,6 @@
           <t>Exploitation research, malware RE, adversary technique talks</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Premier international conference; strong malware and reverse engineering tracks with ransomware family content.</t>
@@ -1746,8 +1696,6 @@
           <t>IR case studies, red/blue team techniques, ransomware response</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>Practitioner-heavy conference with strong IR and blue team focus; good ransomware response content.</t>
@@ -1772,7 +1720,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@SecTorCA</t>
+          <t>https://www.youtube.com/channel/UChoKA8GQo6XIRxJOIDE15oA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1795,8 +1743,6 @@
           <t>Security research talks, IR and threat intelligence sessions</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>Canada's premier security conference; enterprise-focused with solid IR and ransomware response content.</t>
@@ -1844,8 +1790,6 @@
           <t>Security research talks, technical deep dives</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>Regional conference with growing technical depth; useful supplementary coverage.</t>
@@ -1893,16 +1837,14 @@
           <t>Research-heavy talks, vulnerability and exploitation content</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Research-heavy conference; useful for exploitation techniques relevant to ransomware initial access.</t>
+          <t>Research-heavy conference; useful for exploitation techniques relevant to ransomware initial access. [EXCLUDED: no dedicated YouTube channel found via API handle lookup or name search as of 2026-08-11 — likely hosted only on other platforms/conference archives.]</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1942,8 +1884,6 @@
           <t>OT/ICS security talks, ransomware impact on industrial systems</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>DEF CON village focused on ICS/OT; critical for ransomware-on-industrial-infrastructure coverage not found in mainstream channels.</t>
@@ -1991,16 +1931,14 @@
           <t>European security research, malware and threat intelligence talks</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Luxembourg-based European conference; strong malware and ransomware research from European practitioners.</t>
+          <t>Luxembourg-based European conference; strong malware and ransomware research from European practitioners. [EXCLUDED: no dedicated YouTube channel found via API handle lookup or name search as of 2026-08-11 — likely hosted only on other platforms/conference archives.]</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2040,8 +1978,6 @@
           <t>Enterprise security research, Active Directory, network defence</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>German conference; strong Active Directory and enterprise security content highly relevant to ransomware lateral movement.</t>
@@ -2089,8 +2025,6 @@
           <t>Microsoft-hosted security research talks, ransomware defence</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>Microsoft's internal security conference; strong Windows-platform ransomware defence and response content.</t>
@@ -2138,8 +2072,6 @@
           <t>Nation-state actor analysis, ransomware-as-geopolitical-tool</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>Focused on nation-state threats; covers ransomware used as geopolitical instrument (e.g. North Korea, Iran) often absent from other channels.</t>
@@ -2187,8 +2119,6 @@
           <t>Exploitation research, low-level vulnerability analysis</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>Deep exploitation research; useful for understanding vulnerability classes used in ransomware initial access.</t>
@@ -2213,7 +2143,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@Claroty</t>
+          <t>https://www.youtube.com/channel/UC82cIUC3ZzlVjiNvMGe4dHA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2236,8 +2166,6 @@
           <t>OT/ICS threat briefings, ransomware impact on industrial environments</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>OT/ICS security vendor; strong coverage of ransomware hitting manufacturing, energy, and utilities sectors.</t>
@@ -2285,8 +2213,6 @@
           <t>ICS threat intelligence, ransomware in operational technology</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>ICS-focused threat intel vendor; covers ransomware targeting operational technology networks.</t>
@@ -2334,8 +2260,6 @@
           <t>ICS security talks, ransomware impact on critical infrastructure</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>Premier ICS security conference (Dale Peterson); strong content on ransomware disrupting critical infrastructure — Colonial Pipeline-type incidents.</t>
@@ -2383,8 +2307,6 @@
           <t>Ransomware advisories, government guidance, StopRansomware briefings</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>US Cybersecurity and Infrastructure Security Agency; publishes official StopRansomware advisories and briefings — unique government perspective.</t>
@@ -2432,8 +2354,6 @@
           <t>Critical infrastructure defence, air-gap and OT security</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>Air-gap and unidirectional gateway vendor; covers ransomware threat to critical infrastructure from a defence architecture perspective.</t>
@@ -2458,7 +2378,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@RiskyBusiness</t>
+          <t>https://www.youtube.com/channel/UCZzIaWixWHa96R7K4c40_Dg</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2481,8 +2401,6 @@
           <t>Weekly security news podcast, expert interviews on ransomware incidents</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>Top infosec news show (Patrick Gray); ransomware incidents covered in depth with vendor and researcher guests. Lower technical density but strong contextual value.</t>
@@ -2530,8 +2448,6 @@
           <t>Weekly shows with vendor and practitioner guests, threat roundups</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>Long-running show (Paul Asadoorian); high volume with mixed technical depth — good for incident and actor name coverage.</t>
@@ -2556,7 +2472,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@DarknetDiaries</t>
+          <t>https://www.youtube.com/channel/UCMIqrmh2lMdzhlCPK5ahsAg</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2579,8 +2495,6 @@
           <t>Story-driven incident breakdowns, ransomware case narratives</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>Jack Rhysider; narrative-style incident breakdowns including ransomware cases. Lower technical density but strong for actor name and family coverage.</t>
@@ -2605,7 +2519,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@cyb3rops</t>
+          <t>https://www.youtube.com/channel/UC9lFYoA9MAFhnAzX-AtXFxw</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2628,8 +2542,6 @@
           <t>YARA rule writing, Sigma detection, threat hunting</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>Author of YARA and key Sigma rules for ransomware detection; content highly aligned with detection engineering for ransomware IoCs.</t>
@@ -2677,16 +2589,14 @@
           <t>DFIR tooling walkthroughs — KAPE, Timeline Explorer, artefact analysis</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Creator of KAPE and other DFIR tools widely used in ransomware incident response; tooling content directly relevant to ransomware artefact collection.</t>
+          <t>Creator of KAPE and other DFIR tools widely used in ransomware incident response; tooling content directly relevant to ransomware artefact collection. [EXCLUDED: no dedicated YouTube channel found via API handle lookup or name search as of 2026-08-11 — likely hosted only on other platforms/conference archives.]</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2726,8 +2636,6 @@
           <t>SOC training, ransomware investigation labs, blue team walkthroughs</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>SOC training platform with ransomware investigation scenario content; useful for detection and response language coverage.</t>
@@ -2750,17 +2658,11 @@
           <t>Active Countermeasures (already C43)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>— duplicate, already in Batch 1 —</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
           <t>Duplicate check placeholder — remove or replace with new candidate before finalising.</t>
@@ -2808,8 +2710,6 @@
           <t>IR case studies, threat briefings, ransomware response</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>Security consulting firm with dedicated ransomware response practice; regular threat intelligence and IR content.</t>
@@ -2857,8 +2757,6 @@
           <t>Threat intel platform content, actor profiling, IOC analysis</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>TIP vendor with regular threat briefings including ransomware actor and campaign coverage.</t>
@@ -2906,8 +2804,6 @@
           <t>IR case studies, threat briefings, ransomware trends</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>Large security integrator with IR practice; publishes ransomware response and preparedness content.</t>
@@ -2955,8 +2851,6 @@
           <t>Exploitation research, vulnerability analysis, security research talks</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>Pacific-rim conference; strong exploitation and vulnerability research useful for ransomware initial access context.</t>

</xml_diff>